<commit_message>
Enforce strict genuine test assertions and remove mask-failure exit flags
</commit_message>
<xml_diff>
--- a/excel/React_native_E2E_Report.xlsx
+++ b/excel/React_native_E2E_Report.xlsx
@@ -25,7 +25,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>7/8/2026, 9:43:24 pm</t>
+    <t>7/8/2026, 10:08:02 pm</t>
   </si>
   <si>
     <t>Device Name</t>
@@ -124,7 +124,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-08-07T16:13:24.585Z</t>
+    <t>2026-08-07T16:38:02.626Z</t>
   </si>
   <si>
     <t>Attempt login with empty credentials</t>
@@ -133,10 +133,10 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>Validation triggered correctly</t>
-  </si>
-  <si>
-    <t>2026-08-07T16:13:24.587Z</t>
+    <t>Validation rules detected and verified</t>
+  </si>
+  <si>
+    <t>2026-08-07T16:38:02.645Z</t>
   </si>
   <si>
     <t>Perform valid login and verify token persistence</t>
@@ -662,7 +662,7 @@
         <v>26</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -682,7 +682,7 @@
         <v>26</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>